<commit_message>
fix: correção formatação datas - possivelmente responsavel pela troca mes/dia que deu problema
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte.xlsx
+++ b/data/greif/temp/grid_db_suporte.xlsx
@@ -47,25 +47,25 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>EDJANE RODRIGUES DOS SANTOS</t>
-  </si>
-  <si>
-    <t>058.925.079-55</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salva vida emergências médicas </t>
-  </si>
-  <si>
-    <t>u072</t>
-  </si>
-  <si>
-    <t>Dr. Henrique F. Vaz</t>
+    <t>JULIO MARTINS NETO</t>
+  </si>
+  <si>
+    <t>045.154.169-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atendimento on-line </t>
+  </si>
+  <si>
+    <t>M54.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Celso coelho de carvalho </t>
   </si>
   <si>
     <t>PR</t>
   </si>
   <si>
-    <t>CRM-PR 55.550</t>
+    <t>1185853</t>
   </si>
 </sst>
 </file>
@@ -442,16 +442,16 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="32.991943" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="23.422852" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="31.706543" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="16.424561" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -495,10 +495,10 @@
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="7">
-        <v>45964</v>
+        <v>46062</v>
       </c>
       <c r="E2" s="8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
git ignore atualizado + outras mudanças
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte.xlsx
+++ b/data/greif/temp/grid_db_suporte.xlsx
@@ -47,25 +47,25 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>EDJANE RODRIGUES DOS SANTOS</t>
-  </si>
-  <si>
-    <t>058.925.079-55</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salva vida emergências médicas </t>
-  </si>
-  <si>
-    <t>u072</t>
-  </si>
-  <si>
-    <t>Dr. Henrique F. Vaz</t>
+    <t>JULIO MARTINS NETO</t>
+  </si>
+  <si>
+    <t>045.154.169-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atendimento on-line </t>
+  </si>
+  <si>
+    <t>M54.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Celso coelho de carvalho </t>
   </si>
   <si>
     <t>PR</t>
   </si>
   <si>
-    <t>CRM-PR 55.550</t>
+    <t>1185853</t>
   </si>
 </sst>
 </file>
@@ -442,16 +442,16 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="32.991943" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="23.422852" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="31.706543" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="16.424561" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -495,10 +495,10 @@
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="7">
-        <v>45964</v>
+        <v>46062</v>
       </c>
       <c r="E2" s="8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
fix: algumas mudanças e deleções pequenas -> objetivo é estar pronta pra produção
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte.xlsx
+++ b/data/greif/temp/grid_db_suporte.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>Cod Funcionario</t>
   </si>
@@ -47,25 +47,22 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>JULIO MARTINS NETO</t>
-  </si>
-  <si>
-    <t>045.154.169-36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atendimento on-line </t>
-  </si>
-  <si>
-    <t>M54.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Celso coelho de carvalho </t>
-  </si>
-  <si>
-    <t>PR</t>
-  </si>
-  <si>
-    <t>1185853</t>
+    <t>GELSON DA SILVA CEZARIO</t>
+  </si>
+  <si>
+    <t>103.082.337-51</t>
+  </si>
+  <si>
+    <t>Odontovipmaster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabiana de Araújo </t>
+  </si>
+  <si>
+    <t>RJ</t>
+  </si>
+  <si>
+    <t>50780</t>
   </si>
 </sst>
 </file>
@@ -442,14 +439,14 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="22.280273" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="28.135986" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="31.706543" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
@@ -495,7 +492,7 @@
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="7">
-        <v>46062</v>
+        <v>46141</v>
       </c>
       <c r="E2" s="8">
         <v>2</v>
@@ -503,17 +500,15 @@
       <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>